<commit_message>
fix(pro-novinare): vypořádání review Codexu, kolo 1
- Uchazeči: jen žáci základní školy (aspoň jedna denní nezkrácená
  přihláška mimo nástavbu); 13 514 lidí s dálkovým, zkráceným nebo
  nástavbovým studiem se uvádí zvlášť. Deváťáci nepřijatí nikam
  2026: 9 550 z 116 693 (8,2 %), ne 10,2 %.
- Katalog nabídek podle roku z registru, ne applications_2026.json.
- Relativní „loni/letos“ z poznámek veletrhů nahrazeny rokem.
- Bez výrazu „hranice přijetí“ na stránce i v balíčcích.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/pro-novinare/uchazeci-1-kolo-2026.xlsx
+++ b/public/pro-novinare/uchazeci-1-kolo-2026.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
@@ -457,50 +457,57 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Uchazeči, kteří se nedostali na víceleté gymnázium (5. a 7. třída), pokračují na základní škole. Proto se ročníky nesčítají a čísla za 9. třídu se nesmí míchat s víceletými gymnázii.</t>
+          <t>Počítají se uchazeči s aspoň jednou přihláškou do denního nezkráceného studia mimo nástavbu. Vyřazeno: 5468 uchazečů jen s přihláškami na dálkové, kombinované, distanční, večerní nebo zkrácené studium a 8046 jen s přihláškami na nástavbu; nejsou to žáci základní školy.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Kraj je kraj školy, kterou měl uchazeč na přihlášce jako první. Bydliště uchazeče zdroj neuvádí.</t>
+          <t>Uchazeči, kteří se nedostali na víceleté gymnázium (5. a 7. třída), pokračují na základní škole. Proto se ročníky nesčítají a čísla za 9. třídu se nesmí míchat s víceletými gymnázii.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Volba: pořadí oboru na přihlášce. Pořadí na přihlášce šanci na přijetí nemění, škola řadí jen podle svých kritérií.</t>
+          <t>Kraj je kraj školy, kterou měl uchazeč na přihlášce jako první. Bydliště uchazeče zdroj neuvádí.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Přijetí zahrnuje i uchazeče, kteří se přijetí později vzdali: data roku 2026 je nerozlišují.</t>
+          <t>Volba: pořadí oboru na přihlášce. Pořadí na přihlášce šanci na přijetí nemění, škola řadí jen podle svých kritérií.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Nepřijati nikam: v 1. kole se nedostali na žádný obor z přihlášky. Mohli se hlásit do 2. kola; kolik z nich to udělalo, tento balíček neříká.</t>
+          <t>Přijetí zahrnuje i uchazeče, kteří se přijetí později vzdali: data roku 2026 je nerozlišují.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>Nepřijati nikam: v 1. kole se nedostali na žádný obor z přihlášky. Mohli se hlásit do 2. kola; kolik z nich to udělalo, tento balíček neříká.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
           <t>Důvody nepřijetí: nevešli se kvůli kapacitě (splnili požadavky školy, ale jiní měli lepší výsledek), nedosáhli požadavku školy (například minima bodů).</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="inlineStr"/>
-    </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>Zdroj: Přijímačky na školu (prijimackynaskolu.cz), projekt Hlídače státu; zpracování dat CERMAT, MŠMT a vlastní rešerše. Licence CC BY 4.0. https://www.prijimackynaskolu.cz/pro-novinare</t>
         </is>
@@ -614,34 +621,34 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>22541</v>
+        <v>19910</v>
       </c>
       <c r="D2" t="n">
-        <v>17918</v>
+        <v>16178</v>
       </c>
       <c r="E2" t="n">
-        <v>11952</v>
+        <v>10512</v>
       </c>
       <c r="F2" t="n">
-        <v>3850</v>
+        <v>3661</v>
       </c>
       <c r="G2" t="n">
-        <v>2429</v>
+        <v>2371</v>
       </c>
       <c r="H2" t="n">
-        <v>4310</v>
+        <v>3366</v>
       </c>
       <c r="I2" t="n">
-        <v>0.191</v>
+        <v>0.169</v>
       </c>
       <c r="J2" t="n">
-        <v>1170</v>
+        <v>964</v>
       </c>
       <c r="K2" t="n">
-        <v>1334</v>
+        <v>816</v>
       </c>
       <c r="L2" t="n">
-        <v>1806</v>
+        <v>1586</v>
       </c>
       <c r="M2" t="n">
         <v>0</v>
@@ -749,34 +756,34 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>14129</v>
+        <v>12549</v>
       </c>
       <c r="D5" t="n">
-        <v>10156</v>
+        <v>9319</v>
       </c>
       <c r="E5" t="n">
-        <v>9362</v>
+        <v>8258</v>
       </c>
       <c r="F5" t="n">
-        <v>2223</v>
+        <v>2099</v>
       </c>
       <c r="G5" t="n">
-        <v>1197</v>
+        <v>1155</v>
       </c>
       <c r="H5" t="n">
-        <v>1347</v>
+        <v>1037</v>
       </c>
       <c r="I5" t="n">
-        <v>0.095</v>
+        <v>0.083</v>
       </c>
       <c r="J5" t="n">
-        <v>487</v>
+        <v>366</v>
       </c>
       <c r="K5" t="n">
-        <v>372</v>
+        <v>242</v>
       </c>
       <c r="L5" t="n">
-        <v>488</v>
+        <v>429</v>
       </c>
       <c r="M5" t="n">
         <v>0</v>
@@ -884,34 +891,34 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>7920</v>
+        <v>6990</v>
       </c>
       <c r="D8" t="n">
-        <v>5594</v>
+        <v>4907</v>
       </c>
       <c r="E8" t="n">
-        <v>6050</v>
+        <v>5397</v>
       </c>
       <c r="F8" t="n">
-        <v>1014</v>
+        <v>949</v>
       </c>
       <c r="G8" t="n">
-        <v>392</v>
+        <v>372</v>
       </c>
       <c r="H8" t="n">
-        <v>464</v>
+        <v>272</v>
       </c>
       <c r="I8" t="n">
-        <v>0.059</v>
+        <v>0.039</v>
       </c>
       <c r="J8" t="n">
-        <v>211</v>
+        <v>121</v>
       </c>
       <c r="K8" t="n">
-        <v>97</v>
+        <v>52</v>
       </c>
       <c r="L8" t="n">
-        <v>156</v>
+        <v>99</v>
       </c>
       <c r="M8" t="n">
         <v>0</v>
@@ -1019,34 +1026,34 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>2959</v>
+        <v>2801</v>
       </c>
       <c r="D11" t="n">
-        <v>1958</v>
+        <v>1836</v>
       </c>
       <c r="E11" t="n">
-        <v>1974</v>
+        <v>1879</v>
       </c>
       <c r="F11" t="n">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="G11" t="n">
         <v>232</v>
       </c>
       <c r="H11" t="n">
-        <v>287</v>
+        <v>223</v>
       </c>
       <c r="I11" t="n">
-        <v>0.097</v>
+        <v>0.08</v>
       </c>
       <c r="J11" t="n">
-        <v>114</v>
+        <v>96</v>
       </c>
       <c r="K11" t="n">
-        <v>104</v>
+        <v>59</v>
       </c>
       <c r="L11" t="n">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="M11" t="n">
         <v>0</v>
@@ -1154,34 +1161,34 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>6133</v>
+        <v>5254</v>
       </c>
       <c r="D14" t="n">
-        <v>4129</v>
+        <v>3693</v>
       </c>
       <c r="E14" t="n">
-        <v>5009</v>
+        <v>4305</v>
       </c>
       <c r="F14" t="n">
-        <v>593</v>
+        <v>565</v>
       </c>
       <c r="G14" t="n">
-        <v>228</v>
+        <v>216</v>
       </c>
       <c r="H14" t="n">
-        <v>303</v>
+        <v>168</v>
       </c>
       <c r="I14" t="n">
-        <v>0.049</v>
+        <v>0.032</v>
       </c>
       <c r="J14" t="n">
-        <v>136</v>
+        <v>70</v>
       </c>
       <c r="K14" t="n">
-        <v>94</v>
+        <v>42</v>
       </c>
       <c r="L14" t="n">
-        <v>73</v>
+        <v>56</v>
       </c>
       <c r="M14" t="n">
         <v>0</v>
@@ -1289,34 +1296,34 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>6575</v>
+        <v>6065</v>
       </c>
       <c r="D17" t="n">
-        <v>4608</v>
+        <v>4259</v>
       </c>
       <c r="E17" t="n">
-        <v>4718</v>
+        <v>4428</v>
       </c>
       <c r="F17" t="n">
-        <v>900</v>
+        <v>862</v>
       </c>
       <c r="G17" t="n">
-        <v>369</v>
+        <v>357</v>
       </c>
       <c r="H17" t="n">
-        <v>588</v>
+        <v>418</v>
       </c>
       <c r="I17" t="n">
-        <v>0.089</v>
+        <v>0.06900000000000001</v>
       </c>
       <c r="J17" t="n">
-        <v>164</v>
+        <v>103</v>
       </c>
       <c r="K17" t="n">
-        <v>227</v>
+        <v>145</v>
       </c>
       <c r="L17" t="n">
-        <v>197</v>
+        <v>170</v>
       </c>
       <c r="M17" t="n">
         <v>0</v>
@@ -1424,34 +1431,34 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>5422</v>
+        <v>5002</v>
       </c>
       <c r="D20" t="n">
-        <v>3631</v>
+        <v>3256</v>
       </c>
       <c r="E20" t="n">
-        <v>3525</v>
+        <v>3299</v>
       </c>
       <c r="F20" t="n">
-        <v>854</v>
+        <v>835</v>
       </c>
       <c r="G20" t="n">
-        <v>406</v>
+        <v>400</v>
       </c>
       <c r="H20" t="n">
-        <v>637</v>
+        <v>468</v>
       </c>
       <c r="I20" t="n">
-        <v>0.117</v>
+        <v>0.094</v>
       </c>
       <c r="J20" t="n">
-        <v>290</v>
+        <v>206</v>
       </c>
       <c r="K20" t="n">
-        <v>181</v>
+        <v>121</v>
       </c>
       <c r="L20" t="n">
-        <v>166</v>
+        <v>141</v>
       </c>
       <c r="M20" t="n">
         <v>0</v>
@@ -1559,34 +1566,34 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>13093</v>
+        <v>11908</v>
       </c>
       <c r="D23" t="n">
-        <v>9383</v>
+        <v>8487</v>
       </c>
       <c r="E23" t="n">
-        <v>9645</v>
+        <v>8732</v>
       </c>
       <c r="F23" t="n">
-        <v>1850</v>
+        <v>1802</v>
       </c>
       <c r="G23" t="n">
-        <v>812</v>
+        <v>794</v>
       </c>
       <c r="H23" t="n">
-        <v>786</v>
+        <v>580</v>
       </c>
       <c r="I23" t="n">
-        <v>0.06</v>
+        <v>0.049</v>
       </c>
       <c r="J23" t="n">
-        <v>451</v>
+        <v>333</v>
       </c>
       <c r="K23" t="n">
-        <v>156</v>
+        <v>89</v>
       </c>
       <c r="L23" t="n">
-        <v>179</v>
+        <v>158</v>
       </c>
       <c r="M23" t="n">
         <v>0</v>
@@ -1694,34 +1701,34 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>7489</v>
+        <v>6687</v>
       </c>
       <c r="D26" t="n">
-        <v>5239</v>
+        <v>4633</v>
       </c>
       <c r="E26" t="n">
-        <v>5353</v>
+        <v>4845</v>
       </c>
       <c r="F26" t="n">
-        <v>1059</v>
+        <v>987</v>
       </c>
       <c r="G26" t="n">
-        <v>523</v>
+        <v>506</v>
       </c>
       <c r="H26" t="n">
-        <v>554</v>
+        <v>349</v>
       </c>
       <c r="I26" t="n">
-        <v>0.074</v>
+        <v>0.052</v>
       </c>
       <c r="J26" t="n">
-        <v>239</v>
+        <v>181</v>
       </c>
       <c r="K26" t="n">
-        <v>161</v>
+        <v>65</v>
       </c>
       <c r="L26" t="n">
-        <v>154</v>
+        <v>103</v>
       </c>
       <c r="M26" t="n">
         <v>0</v>
@@ -1829,34 +1836,34 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>6753</v>
+        <v>6089</v>
       </c>
       <c r="D29" t="n">
-        <v>4820</v>
+        <v>4449</v>
       </c>
       <c r="E29" t="n">
-        <v>4745</v>
+        <v>4368</v>
       </c>
       <c r="F29" t="n">
-        <v>934</v>
+        <v>911</v>
       </c>
       <c r="G29" t="n">
-        <v>419</v>
+        <v>408</v>
       </c>
       <c r="H29" t="n">
-        <v>655</v>
+        <v>402</v>
       </c>
       <c r="I29" t="n">
-        <v>0.097</v>
+        <v>0.066</v>
       </c>
       <c r="J29" t="n">
-        <v>267</v>
+        <v>136</v>
       </c>
       <c r="K29" t="n">
-        <v>211</v>
+        <v>125</v>
       </c>
       <c r="L29" t="n">
-        <v>177</v>
+        <v>141</v>
       </c>
       <c r="M29" t="n">
         <v>0</v>
@@ -1919,34 +1926,34 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>7281</v>
+        <v>6450</v>
       </c>
       <c r="D31" t="n">
-        <v>5060</v>
+        <v>4438</v>
       </c>
       <c r="E31" t="n">
-        <v>4939</v>
+        <v>4376</v>
       </c>
       <c r="F31" t="n">
-        <v>1105</v>
+        <v>1046</v>
       </c>
       <c r="G31" t="n">
-        <v>623</v>
+        <v>602</v>
       </c>
       <c r="H31" t="n">
-        <v>614</v>
+        <v>426</v>
       </c>
       <c r="I31" t="n">
-        <v>0.08400000000000001</v>
+        <v>0.066</v>
       </c>
       <c r="J31" t="n">
-        <v>270</v>
+        <v>188</v>
       </c>
       <c r="K31" t="n">
-        <v>125</v>
+        <v>77</v>
       </c>
       <c r="L31" t="n">
-        <v>219</v>
+        <v>161</v>
       </c>
       <c r="M31" t="n">
         <v>0</v>
@@ -2054,34 +2061,34 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>12955</v>
+        <v>11662</v>
       </c>
       <c r="D34" t="n">
-        <v>9357</v>
+        <v>8396</v>
       </c>
       <c r="E34" t="n">
-        <v>8585</v>
+        <v>7807</v>
       </c>
       <c r="F34" t="n">
-        <v>1884</v>
+        <v>1819</v>
       </c>
       <c r="G34" t="n">
-        <v>933</v>
+        <v>915</v>
       </c>
       <c r="H34" t="n">
-        <v>1553</v>
+        <v>1121</v>
       </c>
       <c r="I34" t="n">
-        <v>0.12</v>
+        <v>0.096</v>
       </c>
       <c r="J34" t="n">
-        <v>411</v>
+        <v>297</v>
       </c>
       <c r="K34" t="n">
-        <v>545</v>
+        <v>343</v>
       </c>
       <c r="L34" t="n">
-        <v>597</v>
+        <v>481</v>
       </c>
       <c r="M34" t="n">
         <v>0</v>
@@ -2144,34 +2151,34 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>7285</v>
+        <v>6526</v>
       </c>
       <c r="D36" t="n">
-        <v>5599</v>
+        <v>5000</v>
       </c>
       <c r="E36" t="n">
-        <v>5224</v>
+        <v>4715</v>
       </c>
       <c r="F36" t="n">
-        <v>1111</v>
+        <v>1043</v>
       </c>
       <c r="G36" t="n">
-        <v>483</v>
+        <v>465</v>
       </c>
       <c r="H36" t="n">
-        <v>467</v>
+        <v>303</v>
       </c>
       <c r="I36" t="n">
-        <v>0.064</v>
+        <v>0.046</v>
       </c>
       <c r="J36" t="n">
-        <v>275</v>
+        <v>191</v>
       </c>
       <c r="K36" t="n">
-        <v>87</v>
+        <v>31</v>
       </c>
       <c r="L36" t="n">
-        <v>105</v>
+        <v>81</v>
       </c>
       <c r="M36" t="n">
         <v>0</v>
@@ -2279,34 +2286,34 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>9672</v>
+        <v>8800</v>
       </c>
       <c r="D39" t="n">
-        <v>6328</v>
+        <v>5700</v>
       </c>
       <c r="E39" t="n">
-        <v>7529</v>
+        <v>6997</v>
       </c>
       <c r="F39" t="n">
-        <v>1027</v>
+        <v>989</v>
       </c>
       <c r="G39" t="n">
-        <v>404</v>
+        <v>397</v>
       </c>
       <c r="H39" t="n">
-        <v>712</v>
+        <v>417</v>
       </c>
       <c r="I39" t="n">
-        <v>0.074</v>
+        <v>0.047</v>
       </c>
       <c r="J39" t="n">
-        <v>266</v>
+        <v>96</v>
       </c>
       <c r="K39" t="n">
-        <v>249</v>
+        <v>156</v>
       </c>
       <c r="L39" t="n">
-        <v>197</v>
+        <v>165</v>
       </c>
       <c r="M39" t="n">
         <v>0</v>
@@ -2510,34 +2517,34 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>130207</v>
+        <v>116693</v>
       </c>
       <c r="D2" t="n">
-        <v>93780</v>
+        <v>84551</v>
       </c>
       <c r="E2" t="n">
-        <v>88610</v>
+        <v>79918</v>
       </c>
       <c r="F2" t="n">
-        <v>18870</v>
+        <v>18035</v>
       </c>
       <c r="G2" t="n">
-        <v>9450</v>
+        <v>9190</v>
       </c>
       <c r="H2" t="n">
-        <v>13277</v>
+        <v>9550</v>
       </c>
       <c r="I2" t="n">
-        <v>0.102</v>
+        <v>0.082</v>
       </c>
       <c r="J2" t="n">
-        <v>4751</v>
+        <v>3348</v>
       </c>
       <c r="K2" t="n">
-        <v>3943</v>
+        <v>2363</v>
       </c>
       <c r="L2" t="n">
-        <v>4583</v>
+        <v>3839</v>
       </c>
       <c r="M2" t="n">
         <v>0</v>

</xml_diff>